<commit_message>
remove old model files
</commit_message>
<xml_diff>
--- a/Model objective analysis/Capacity increase/L shape base model 35 scenarios/L_Shape_base_35_tender_fixed.xlsx
+++ b/Model objective analysis/Capacity increase/L shape base model 35 scenarios/L_Shape_base_35_tender_fixed.xlsx
@@ -452,7 +452,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -460,10 +460,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -473,7 +473,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -481,10 +481,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -515,7 +515,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -526,7 +526,7 @@
         <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -536,7 +536,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D6" t="n">
         <v>10</v>
@@ -809,7 +809,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -817,7 +817,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D19" t="n">
         <v>10</v>
@@ -830,7 +830,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -841,7 +841,7 @@
         <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -935,7 +935,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -943,7 +943,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D25" t="n">
         <v>10</v>
@@ -956,7 +956,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -967,7 +967,7 @@
         <v>2</v>
       </c>
       <c r="D26" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1061,7 +1061,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>416</v>
+        <v>412</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1069,7 +1069,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D31" t="n">
         <v>10</v>
@@ -1082,7 +1082,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1093,7 +1093,7 @@
         <v>2</v>
       </c>
       <c r="D32" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>

</xml_diff>